<commit_message>
Worked on the analysis of the results.
</commit_message>
<xml_diff>
--- a/results/multi_size_training/plots/indist/06_gap_table.xlsx
+++ b/results/multi_size_training/plots/indist/06_gap_table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,7 +473,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gap %</t>
+          <t>Optimal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -573,8 +573,10 @@
       <c r="B4" t="n">
         <v>122.97</v>
       </c>
-      <c r="C4" t="n">
-        <v>0</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>100/100</t>
+        </is>
       </c>
       <c r="D4" t="n">
         <v>143.76</v>
@@ -628,589 +630,738 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>20x10</t>
+          <t>20x5</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>191.07</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
+        <v>187.76</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>205.63</v>
+        <v>204.67</v>
       </c>
       <c r="E5" t="n">
-        <v>7.616459773523411</v>
+        <v>8.999971598759302</v>
       </c>
       <c r="F5" t="n">
-        <v>274.66</v>
+        <v>252.72</v>
       </c>
       <c r="G5" t="n">
-        <v>43.79654530189305</v>
+        <v>34.75601897092313</v>
       </c>
       <c r="H5" t="n">
-        <v>209.4</v>
+        <v>207.78</v>
       </c>
       <c r="I5" t="n">
-        <v>9.600363004258304</v>
+        <v>10.66436616957846</v>
       </c>
       <c r="J5" t="n">
-        <v>253.12</v>
+        <v>229.01</v>
       </c>
       <c r="K5" t="n">
-        <v>32.5293743494318</v>
+        <v>22.0552851842065</v>
       </c>
       <c r="L5" t="n">
-        <v>216.1466666666667</v>
+        <v>210.3033333333333</v>
       </c>
       <c r="M5" t="n">
-        <v>13.13592882141409</v>
+        <v>12.03509093680163</v>
       </c>
       <c r="N5" t="n">
-        <v>215.28</v>
+        <v>205.76</v>
       </c>
       <c r="O5" t="n">
-        <v>12.68285283446519</v>
+        <v>9.594438829732708</v>
       </c>
       <c r="P5" t="n">
-        <v>217.89</v>
+        <v>210.2666666666667</v>
       </c>
       <c r="Q5" t="n">
-        <v>14.05021358315696</v>
+        <v>12.00845150310242</v>
       </c>
       <c r="R5" t="n">
-        <v>218.1933333333334</v>
+        <v>206.96</v>
       </c>
       <c r="S5" t="n">
-        <v>14.21021020904402</v>
+        <v>10.23987054644589</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20x20</t>
+          <t>20x10</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>236.01</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
+        <v>191.07</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>268.13</v>
+        <v>205.63</v>
       </c>
       <c r="E6" t="n">
-        <v>13.60793096210382</v>
+        <v>7.616459773523411</v>
       </c>
       <c r="F6" t="n">
-        <v>309.95</v>
+        <v>274.66</v>
       </c>
       <c r="G6" t="n">
-        <v>31.46352298728664</v>
+        <v>43.79654530189305</v>
       </c>
       <c r="H6" t="n">
-        <v>269.62</v>
+        <v>209.4</v>
       </c>
       <c r="I6" t="n">
-        <v>14.28998860359803</v>
+        <v>9.600363004258304</v>
       </c>
       <c r="J6" t="n">
-        <v>280.47</v>
+        <v>253.12</v>
       </c>
       <c r="K6" t="n">
-        <v>18.91611889186488</v>
+        <v>32.5293743494318</v>
       </c>
       <c r="L6" t="n">
-        <v>283.7333333333333</v>
+        <v>216.1466666666667</v>
       </c>
       <c r="M6" t="n">
-        <v>20.23050881558559</v>
+        <v>13.13592882141409</v>
       </c>
       <c r="N6" t="n">
-        <v>272.32</v>
+        <v>215.28</v>
       </c>
       <c r="O6" t="n">
-        <v>15.45229074027858</v>
+        <v>12.68285283446519</v>
       </c>
       <c r="P6" t="n">
-        <v>287.9066666666667</v>
+        <v>217.89</v>
       </c>
       <c r="Q6" t="n">
-        <v>22.00571204999832</v>
+        <v>14.05021358315696</v>
       </c>
       <c r="R6" t="n">
-        <v>272.68</v>
+        <v>218.1933333333334</v>
       </c>
       <c r="S6" t="n">
-        <v>15.59941577048973</v>
+        <v>14.21021020904402</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>20x30</t>
+          <t>20x20</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>336.33</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
+        <v>236.01</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>70/100</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>378.18</v>
+        <v>268.13</v>
       </c>
       <c r="E7" t="n">
-        <v>12.49150025440501</v>
+        <v>13.60793096210382</v>
       </c>
       <c r="F7" t="n">
-        <v>382.24</v>
+        <v>309.95</v>
       </c>
       <c r="G7" t="n">
-        <v>13.75872382001964</v>
+        <v>31.46352298728664</v>
       </c>
       <c r="H7" t="n">
-        <v>378.07</v>
+        <v>269.62</v>
       </c>
       <c r="I7" t="n">
-        <v>12.48179703821259</v>
+        <v>14.28998860359803</v>
       </c>
       <c r="J7" t="n">
-        <v>383.67</v>
+        <v>280.47</v>
       </c>
       <c r="K7" t="n">
-        <v>14.1414746903501</v>
+        <v>18.91611889186488</v>
       </c>
       <c r="L7" t="n">
-        <v>402.26</v>
+        <v>283.7333333333333</v>
       </c>
       <c r="M7" t="n">
-        <v>19.65838228725153</v>
+        <v>20.23050881558559</v>
       </c>
       <c r="N7" t="n">
-        <v>387.6866666666667</v>
+        <v>272.32</v>
       </c>
       <c r="O7" t="n">
-        <v>15.3368982221098</v>
+        <v>15.45229074027858</v>
       </c>
       <c r="P7" t="n">
-        <v>410.43</v>
+        <v>287.9066666666667</v>
       </c>
       <c r="Q7" t="n">
-        <v>22.06246336550391</v>
+        <v>22.00571204999832</v>
       </c>
       <c r="R7" t="n">
-        <v>387.91</v>
+        <v>272.68</v>
       </c>
       <c r="S7" t="n">
-        <v>15.40225684917877</v>
+        <v>15.59941577048973</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>30x10</t>
+          <t>20x30</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>280.48</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
+        <v>336.33</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>100/100</t>
+        </is>
       </c>
       <c r="D8" t="n">
-        <v>296.93</v>
+        <v>378.18</v>
       </c>
       <c r="E8" t="n">
-        <v>5.872639960424017</v>
+        <v>12.49150025440501</v>
       </c>
       <c r="F8" t="n">
-        <v>367.62</v>
+        <v>382.24</v>
       </c>
       <c r="G8" t="n">
-        <v>31.11601636634635</v>
+        <v>13.75872382001964</v>
       </c>
       <c r="H8" t="n">
-        <v>301.04</v>
+        <v>378.07</v>
       </c>
       <c r="I8" t="n">
-        <v>7.344345695569262</v>
+        <v>12.48179703821259</v>
       </c>
       <c r="J8" t="n">
-        <v>348.55</v>
+        <v>383.67</v>
       </c>
       <c r="K8" t="n">
-        <v>24.33529811995803</v>
+        <v>14.1414746903501</v>
       </c>
       <c r="L8" t="n">
-        <v>312.9966666666667</v>
+        <v>402.26</v>
       </c>
       <c r="M8" t="n">
-        <v>11.60214043028049</v>
+        <v>19.65838228725153</v>
       </c>
       <c r="N8" t="n">
-        <v>312.36</v>
+        <v>387.6866666666667</v>
       </c>
       <c r="O8" t="n">
-        <v>11.37737424769339</v>
+        <v>15.3368982221098</v>
       </c>
       <c r="P8" t="n">
-        <v>314.55</v>
+        <v>410.43</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.16299788152144</v>
+        <v>22.06246336550391</v>
       </c>
       <c r="R8" t="n">
-        <v>315.66</v>
+        <v>387.91</v>
       </c>
       <c r="S8" t="n">
-        <v>12.55861960216554</v>
+        <v>15.40225684917877</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>40x10</t>
+          <t>30x10</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>374.74</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
+        <v>280.48</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
       </c>
       <c r="D9" t="n">
-        <v>394.16</v>
+        <v>296.93</v>
       </c>
       <c r="E9" t="n">
-        <v>5.184797135785824</v>
+        <v>5.872639960424017</v>
       </c>
       <c r="F9" t="n">
-        <v>458.42</v>
+        <v>367.62</v>
       </c>
       <c r="G9" t="n">
-        <v>22.32034295266108</v>
+        <v>31.11601636634635</v>
       </c>
       <c r="H9" t="n">
-        <v>399.74</v>
+        <v>301.04</v>
       </c>
       <c r="I9" t="n">
-        <v>6.688421744719647</v>
+        <v>7.344345695569262</v>
       </c>
       <c r="J9" t="n">
-        <v>446.58</v>
+        <v>348.55</v>
       </c>
       <c r="K9" t="n">
-        <v>19.18153907473868</v>
+        <v>24.33529811995803</v>
       </c>
       <c r="L9" t="n">
-        <v>416.3633333333333</v>
+        <v>312.9966666666667</v>
       </c>
       <c r="M9" t="n">
-        <v>11.11363760777877</v>
+        <v>11.60214043028049</v>
       </c>
       <c r="N9" t="n">
-        <v>415.3833333333334</v>
+        <v>312.36</v>
       </c>
       <c r="O9" t="n">
-        <v>10.8531318360499</v>
+        <v>11.37737424769339</v>
       </c>
       <c r="P9" t="n">
-        <v>417.9633333333334</v>
+        <v>314.55</v>
       </c>
       <c r="Q9" t="n">
-        <v>11.54191712574671</v>
+        <v>12.16299788152144</v>
       </c>
       <c r="R9" t="n">
-        <v>418.3366666666666</v>
+        <v>315.66</v>
       </c>
       <c r="S9" t="n">
-        <v>11.63984162885008</v>
+        <v>12.55861960216554</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>50x10</t>
+          <t>40x10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>470.37</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
+        <v>374.74</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
       </c>
       <c r="D10" t="n">
-        <v>491.14</v>
+        <v>394.16</v>
       </c>
       <c r="E10" t="n">
-        <v>4.427720269966894</v>
+        <v>5.184797135785824</v>
       </c>
       <c r="F10" t="n">
-        <v>556</v>
+        <v>458.42</v>
       </c>
       <c r="G10" t="n">
-        <v>18.21148140363564</v>
+        <v>22.32034295266108</v>
       </c>
       <c r="H10" t="n">
-        <v>497.29</v>
+        <v>399.74</v>
       </c>
       <c r="I10" t="n">
-        <v>5.741124533801951</v>
+        <v>6.688421744719647</v>
       </c>
       <c r="J10" t="n">
-        <v>545.6</v>
+        <v>446.58</v>
       </c>
       <c r="K10" t="n">
-        <v>16.04498951550163</v>
+        <v>19.18153907473868</v>
       </c>
       <c r="L10" t="n">
-        <v>520.3233333333334</v>
+        <v>416.3633333333333</v>
       </c>
       <c r="M10" t="n">
-        <v>10.6377567976346</v>
+        <v>11.11363760777877</v>
       </c>
       <c r="N10" t="n">
-        <v>519.2666666666668</v>
+        <v>415.3833333333334</v>
       </c>
       <c r="O10" t="n">
-        <v>10.41060306605543</v>
+        <v>10.8531318360499</v>
       </c>
       <c r="P10" t="n">
-        <v>521.8000000000001</v>
+        <v>417.9633333333334</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.95268426842517</v>
+        <v>11.54191712574671</v>
       </c>
       <c r="R10" t="n">
-        <v>522.1</v>
+        <v>418.3366666666666</v>
       </c>
       <c r="S10" t="n">
-        <v>11.01374758992847</v>
+        <v>11.63984162885008</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>100x10</t>
+          <t>50x10</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>939.48</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
+        <v>470.37</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
       </c>
       <c r="D11" t="n">
-        <v>974.36</v>
+        <v>491.14</v>
       </c>
       <c r="E11" t="n">
-        <v>3.733694651835385</v>
+        <v>4.427720269966894</v>
       </c>
       <c r="F11" t="n">
-        <v>1018.14</v>
+        <v>556</v>
       </c>
       <c r="G11" t="n">
-        <v>8.401298237136134</v>
+        <v>18.21148140363564</v>
       </c>
       <c r="H11" t="n">
-        <v>981.9400000000001</v>
+        <v>497.29</v>
       </c>
       <c r="I11" t="n">
-        <v>4.540170788544645</v>
+        <v>5.741124533801951</v>
       </c>
       <c r="J11" t="n">
-        <v>1031.4</v>
+        <v>545.6</v>
       </c>
       <c r="K11" t="n">
-        <v>9.802495597259604</v>
+        <v>16.04498951550163</v>
       </c>
       <c r="L11" t="n">
-        <v>1032.01</v>
+        <v>520.3233333333334</v>
       </c>
       <c r="M11" t="n">
-        <v>9.872951466825699</v>
+        <v>10.6377567976346</v>
       </c>
       <c r="N11" t="n">
-        <v>1028.55</v>
+        <v>519.2666666666668</v>
       </c>
       <c r="O11" t="n">
-        <v>9.503885375620882</v>
+        <v>10.41060306605543</v>
       </c>
       <c r="P11" t="n">
-        <v>1032.956666666667</v>
+        <v>521.8000000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>9.972597671195588</v>
+        <v>10.95268426842517</v>
       </c>
       <c r="R11" t="n">
-        <v>1032.4</v>
+        <v>522.1</v>
       </c>
       <c r="S11" t="n">
-        <v>9.914630261099992</v>
+        <v>11.01374758992847</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>200x10</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+          <t>100x10</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>939.48</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
+      </c>
       <c r="D12" t="n">
-        <v>1951.78</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
+        <v>974.36</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.733694651835385</v>
+      </c>
       <c r="F12" t="n">
-        <v>1925.66</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+        <v>1018.14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8.401298237136134</v>
+      </c>
       <c r="H12" t="n">
-        <v>1961.38</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
+        <v>981.9400000000001</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.540170788544645</v>
+      </c>
       <c r="J12" t="n">
-        <v>2012.16</v>
-      </c>
-      <c r="K12" t="inlineStr"/>
+        <v>1031.4</v>
+      </c>
+      <c r="K12" t="n">
+        <v>9.802495597259604</v>
+      </c>
       <c r="L12" t="n">
-        <v>2065</v>
-      </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
+        <v>1032.01</v>
+      </c>
+      <c r="M12" t="n">
+        <v>9.872951466825699</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1028.55</v>
+      </c>
+      <c r="O12" t="n">
+        <v>9.503885375620882</v>
+      </c>
       <c r="P12" t="n">
-        <v>2070.426666666667</v>
-      </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+        <v>1032.956666666667</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>9.972597671195588</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1032.4</v>
+      </c>
+      <c r="S12" t="n">
+        <v>9.914630261099992</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>edata</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+          <t>200x10</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1919.26</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>0/100</t>
+        </is>
+      </c>
       <c r="D13" t="n">
-        <v>2045.121212121212</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
+        <v>1951.78</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.741014237905788</v>
+      </c>
       <c r="F13" t="n">
-        <v>2045.257575757576</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+        <v>1925.66</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.3834534570887586</v>
+      </c>
       <c r="H13" t="n">
-        <v>2093.863636363636</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
+        <v>1961.38</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.243899165510101</v>
+      </c>
       <c r="J13" t="n">
-        <v>2243.712121212121</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
+        <v>2012.16</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4.886161473592739</v>
+      </c>
       <c r="L13" t="n">
-        <v>2059.691919191919</v>
-      </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
-        <v>1880.575757575757</v>
-      </c>
+        <v>2065</v>
+      </c>
+      <c r="M13" t="n">
+        <v>7.645481816986436</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
-        <v>2052.969696969697</v>
-      </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="n">
-        <v>1886.232323232323</v>
-      </c>
+        <v>2070.426666666667</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>7.925908602781337</v>
+      </c>
+      <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>rdata</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>edata</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1697.030303030303</v>
+      </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="n">
-        <v>1687.439393939394</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
+        <v>2045.121212121212</v>
+      </c>
+      <c r="E14" t="n">
+        <v>17.04347759731398</v>
+      </c>
       <c r="F14" t="n">
-        <v>1808.015151515152</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
+        <v>2045.257575757576</v>
+      </c>
+      <c r="G14" t="n">
+        <v>23.06149594518934</v>
+      </c>
       <c r="H14" t="n">
-        <v>1702.651515151515</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>2093.863636363636</v>
+      </c>
+      <c r="I14" t="n">
+        <v>19.55408016987395</v>
+      </c>
       <c r="J14" t="n">
-        <v>1820.106060606061</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
+        <v>2243.712121212121</v>
+      </c>
+      <c r="K14" t="n">
+        <v>32.4150004948589</v>
+      </c>
       <c r="L14" t="n">
-        <v>1646.686868686869</v>
-      </c>
-      <c r="M14" t="inlineStr"/>
+        <v>2059.691919191919</v>
+      </c>
+      <c r="M14" t="n">
+        <v>18.82935978663038</v>
+      </c>
       <c r="N14" t="n">
-        <v>1536.212121212121</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>1880.575757575757</v>
+      </c>
+      <c r="O14" t="n">
+        <v>10.74763893992157</v>
+      </c>
       <c r="P14" t="n">
-        <v>1675.111111111111</v>
-      </c>
-      <c r="Q14" t="inlineStr"/>
+        <v>2052.969696969697</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>19.45756219547593</v>
+      </c>
       <c r="R14" t="n">
-        <v>1551.808080808081</v>
-      </c>
-      <c r="S14" t="inlineStr"/>
+        <v>1886.232323232323</v>
+      </c>
+      <c r="S14" t="n">
+        <v>11.14232811568861</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>vdata</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>rdata</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1426.378787878788</v>
+      </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="n">
+        <v>1687.439393939394</v>
+      </c>
+      <c r="E15" t="n">
+        <v>14.46267902354886</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1808.015151515152</v>
+      </c>
+      <c r="G15" t="n">
+        <v>26.46372593116812</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1702.651515151515</v>
+      </c>
+      <c r="I15" t="n">
+        <v>16.3433911190802</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1820.106060606061</v>
+      </c>
+      <c r="K15" t="n">
+        <v>27.72702408777951</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1646.686868686869</v>
+      </c>
+      <c r="M15" t="n">
+        <v>14.29071234468039</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1536.212121212121</v>
+      </c>
+      <c r="O15" t="n">
+        <v>8.545225925703901</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1675.111111111111</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>16.41571584755398</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1551.808080808081</v>
+      </c>
+      <c r="S15" t="n">
+        <v>9.632456303122041</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>vdata</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1365.939393939394</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
         <v>1442.560606060606</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="n">
+      <c r="E16" t="n">
+        <v>2.976799113029442</v>
+      </c>
+      <c r="F16" t="n">
         <v>1617.121212121212</v>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
+      <c r="G16" t="n">
+        <v>15.23668765513237</v>
+      </c>
+      <c r="H16" t="n">
         <v>1514.530303030303</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="n">
+      <c r="I16" t="n">
+        <v>5.698985457182911</v>
+      </c>
+      <c r="J16" t="n">
         <v>1639.787878787879</v>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="n">
+      <c r="K16" t="n">
+        <v>15.60004565321777</v>
+      </c>
+      <c r="L16" t="n">
         <v>1446.89898989899</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
+      <c r="M16" t="n">
+        <v>4.9061401731834</v>
+      </c>
+      <c r="N16" t="n">
         <v>1401.434343434343</v>
       </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="n">
+      <c r="O16" t="n">
+        <v>1.94624465131096</v>
+      </c>
+      <c r="P16" t="n">
         <v>1465.565656565657</v>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="n">
+      <c r="Q16" t="n">
+        <v>5.890554270199721</v>
+      </c>
+      <c r="R16" t="n">
         <v>1409.828282828283</v>
       </c>
-      <c r="S15" t="inlineStr"/>
+      <c r="S16" t="n">
+        <v>2.43977599899095</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Working on plots of sagc.
</commit_message>
<xml_diff>
--- a/results/multi_size_training/plots/indist/06_gap_table.xlsx
+++ b/results/multi_size_training/plots/indist/06_gap_table.xlsx
@@ -1193,56 +1193,60 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1697.030303030303</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
+        <v>1696.969696969697</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>59/66</t>
+        </is>
+      </c>
       <c r="D14" t="n">
         <v>2045.121212121212</v>
       </c>
       <c r="E14" t="n">
-        <v>17.04347759731398</v>
+        <v>17.05912655834206</v>
       </c>
       <c r="F14" t="n">
         <v>2045.257575757576</v>
       </c>
       <c r="G14" t="n">
-        <v>23.06149594518934</v>
+        <v>23.08042101648029</v>
       </c>
       <c r="H14" t="n">
         <v>2093.863636363636</v>
       </c>
       <c r="I14" t="n">
-        <v>19.55408016987395</v>
+        <v>19.56883810334718</v>
       </c>
       <c r="J14" t="n">
         <v>2243.712121212121</v>
       </c>
       <c r="K14" t="n">
-        <v>32.4150004948589</v>
+        <v>32.43358151878979</v>
       </c>
       <c r="L14" t="n">
         <v>2059.691919191919</v>
       </c>
       <c r="M14" t="n">
-        <v>18.82935978663038</v>
+        <v>18.84398383454566</v>
       </c>
       <c r="N14" t="n">
         <v>1880.575757575757</v>
       </c>
       <c r="O14" t="n">
-        <v>10.74763893992157</v>
+        <v>10.7619285440672</v>
       </c>
       <c r="P14" t="n">
         <v>2052.969696969697</v>
       </c>
       <c r="Q14" t="n">
-        <v>19.45756219547593</v>
+        <v>19.47298567741927</v>
       </c>
       <c r="R14" t="n">
         <v>1886.232323232323</v>
       </c>
       <c r="S14" t="n">
-        <v>11.14232811568861</v>
+        <v>11.15687375823421</v>
       </c>
     </row>
     <row r="15">
@@ -1252,56 +1256,60 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1426.378787878788</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
+        <v>1426.909090909091</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>34/66</t>
+        </is>
+      </c>
       <c r="D15" t="n">
         <v>1687.439393939394</v>
       </c>
       <c r="E15" t="n">
-        <v>14.46267902354886</v>
+        <v>14.4416374269675</v>
       </c>
       <c r="F15" t="n">
         <v>1808.015151515152</v>
       </c>
       <c r="G15" t="n">
-        <v>26.46372593116812</v>
+        <v>26.45123122328132</v>
       </c>
       <c r="H15" t="n">
         <v>1702.651515151515</v>
       </c>
       <c r="I15" t="n">
-        <v>16.3433911190802</v>
+        <v>16.32245045142188</v>
       </c>
       <c r="J15" t="n">
         <v>1820.106060606061</v>
       </c>
       <c r="K15" t="n">
-        <v>27.72702408777951</v>
+        <v>27.70990812434014</v>
       </c>
       <c r="L15" t="n">
         <v>1646.686868686869</v>
       </c>
       <c r="M15" t="n">
-        <v>14.29071234468039</v>
+        <v>14.27158975841281</v>
       </c>
       <c r="N15" t="n">
         <v>1536.212121212121</v>
       </c>
       <c r="O15" t="n">
-        <v>8.545225925703901</v>
+        <v>8.525761868986047</v>
       </c>
       <c r="P15" t="n">
         <v>1675.111111111111</v>
       </c>
       <c r="Q15" t="n">
-        <v>16.41571584755398</v>
+        <v>16.39825270562874</v>
       </c>
       <c r="R15" t="n">
         <v>1551.808080808081</v>
       </c>
       <c r="S15" t="n">
-        <v>9.632456303122041</v>
+        <v>9.61345261347531</v>
       </c>
     </row>
     <row r="16">
@@ -1311,56 +1319,60 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1365.939393939394</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
+        <v>1366.984848484848</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>27/66</t>
+        </is>
+      </c>
       <c r="D16" t="n">
         <v>1442.560606060606</v>
       </c>
       <c r="E16" t="n">
-        <v>2.976799113029442</v>
+        <v>2.796517177892701</v>
       </c>
       <c r="F16" t="n">
         <v>1617.121212121212</v>
       </c>
       <c r="G16" t="n">
-        <v>15.23668765513237</v>
+        <v>15.025528413241</v>
       </c>
       <c r="H16" t="n">
         <v>1514.530303030303</v>
       </c>
       <c r="I16" t="n">
-        <v>5.698985457182911</v>
+        <v>5.51328268184553</v>
       </c>
       <c r="J16" t="n">
         <v>1639.787878787879</v>
       </c>
       <c r="K16" t="n">
-        <v>15.60004565321777</v>
+        <v>15.36170167065717</v>
       </c>
       <c r="L16" t="n">
         <v>1446.89898989899</v>
       </c>
       <c r="M16" t="n">
-        <v>4.9061401731834</v>
+        <v>4.723600580253306</v>
       </c>
       <c r="N16" t="n">
         <v>1401.434343434343</v>
       </c>
       <c r="O16" t="n">
-        <v>1.94624465131096</v>
+        <v>1.764161059546347</v>
       </c>
       <c r="P16" t="n">
         <v>1465.565656565657</v>
       </c>
       <c r="Q16" t="n">
-        <v>5.890554270199721</v>
+        <v>5.70666897870947</v>
       </c>
       <c r="R16" t="n">
         <v>1409.828282828283</v>
       </c>
       <c r="S16" t="n">
-        <v>2.43977599899095</v>
+        <v>2.256464382135027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjusted the analysis of the multi size training experiment.
</commit_message>
<xml_diff>
--- a/results/multi_size_training/plots/indist/06_gap_table.xlsx
+++ b/results/multi_size_training/plots/indist/06_gap_table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:W16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,22 +445,32 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>SAGC (Greedy)</t>
+          <t>Song+SAGC (multi size) (Greedy)</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>SAGC (Sampling)</t>
+          <t>Song+SAGC (multi size) (Sampling)</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>NoPooling (Greedy)</t>
+          <t>Song (multi size) (Greedy)</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>NoPooling (Sampling)</t>
+          <t>Song (multi size) (Sampling)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Song+SAGC (20x10) (Greedy)</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Song+SAGC (20x10) (Sampling)</t>
         </is>
       </c>
     </row>
@@ -556,6 +566,26 @@
           <t>Gap %</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Makespan</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Gap %</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Makespan</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Gap %</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -626,6 +656,18 @@
       <c r="S4" t="n">
         <v>12.43588190529337</v>
       </c>
+      <c r="T4" t="n">
+        <v>146.3133333333333</v>
+      </c>
+      <c r="U4" t="n">
+        <v>19.2459666998774</v>
+      </c>
+      <c r="V4" t="n">
+        <v>137.3066666666666</v>
+      </c>
+      <c r="W4" t="n">
+        <v>11.87363193442794</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -689,6 +731,18 @@
       <c r="S5" t="n">
         <v>10.23987054644589</v>
       </c>
+      <c r="T5" t="n">
+        <v>209.0433333333333</v>
+      </c>
+      <c r="U5" t="n">
+        <v>11.34286698090205</v>
+      </c>
+      <c r="V5" t="n">
+        <v>205.3333333333333</v>
+      </c>
+      <c r="W5" t="n">
+        <v>9.374558930109869</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -752,6 +806,18 @@
       <c r="S6" t="n">
         <v>14.21021020904402</v>
       </c>
+      <c r="T6" t="n">
+        <v>216.0733333333334</v>
+      </c>
+      <c r="U6" t="n">
+        <v>13.10026980466686</v>
+      </c>
+      <c r="V6" t="n">
+        <v>214.64</v>
+      </c>
+      <c r="W6" t="n">
+        <v>12.34636120856059</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -815,6 +881,18 @@
       <c r="S7" t="n">
         <v>15.59941577048973</v>
       </c>
+      <c r="T7" t="n">
+        <v>282.56</v>
+      </c>
+      <c r="U7" t="n">
+        <v>19.75993481082608</v>
+      </c>
+      <c r="V7" t="n">
+        <v>272.0066666666667</v>
+      </c>
+      <c r="W7" t="n">
+        <v>15.31616154695402</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -878,6 +956,18 @@
       <c r="S8" t="n">
         <v>15.40225684917877</v>
       </c>
+      <c r="T8" t="n">
+        <v>398.6766666666667</v>
+      </c>
+      <c r="U8" t="n">
+        <v>18.58622754871766</v>
+      </c>
+      <c r="V8" t="n">
+        <v>387.79</v>
+      </c>
+      <c r="W8" t="n">
+        <v>15.36314380835855</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -941,6 +1031,18 @@
       <c r="S9" t="n">
         <v>12.55861960216554</v>
       </c>
+      <c r="T9" t="n">
+        <v>314</v>
+      </c>
+      <c r="U9" t="n">
+        <v>11.96361244766874</v>
+      </c>
+      <c r="V9" t="n">
+        <v>312.0466666666667</v>
+      </c>
+      <c r="W9" t="n">
+        <v>11.26646045675859</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1004,6 +1106,18 @@
       <c r="S10" t="n">
         <v>11.63984162885008</v>
       </c>
+      <c r="T10" t="n">
+        <v>416.7033333333334</v>
+      </c>
+      <c r="U10" t="n">
+        <v>11.20688121502601</v>
+      </c>
+      <c r="V10" t="n">
+        <v>414.46</v>
+      </c>
+      <c r="W10" t="n">
+        <v>10.60627822529645</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1067,6 +1181,18 @@
       <c r="S11" t="n">
         <v>11.01374758992847</v>
       </c>
+      <c r="T11" t="n">
+        <v>520.4400000000001</v>
+      </c>
+      <c r="U11" t="n">
+        <v>10.663118187697</v>
+      </c>
+      <c r="V11" t="n">
+        <v>518.1866666666667</v>
+      </c>
+      <c r="W11" t="n">
+        <v>10.18071852800368</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1129,6 +1255,18 @@
       </c>
       <c r="S12" t="n">
         <v>9.914630261099992</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1030.38</v>
+      </c>
+      <c r="U12" t="n">
+        <v>9.699003941397407</v>
+      </c>
+      <c r="V12" t="n">
+        <v>1026.926666666667</v>
+      </c>
+      <c r="W12" t="n">
+        <v>9.331395331314717</v>
       </c>
     </row>
     <row r="13">
@@ -1185,6 +1323,18 @@
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>2061.573333333333</v>
+      </c>
+      <c r="U13" t="n">
+        <v>7.465801894582587</v>
+      </c>
+      <c r="V13" t="n">
+        <v>2056.106666666667</v>
+      </c>
+      <c r="W13" t="n">
+        <v>7.180994827343792</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1248,6 +1398,18 @@
       <c r="S14" t="n">
         <v>11.15687375823421</v>
       </c>
+      <c r="T14" t="n">
+        <v>2038.075757575757</v>
+      </c>
+      <c r="U14" t="n">
+        <v>18.54220570473099</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1884.010101010101</v>
+      </c>
+      <c r="W14" t="n">
+        <v>10.68217369100824</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1311,6 +1473,18 @@
       <c r="S15" t="n">
         <v>9.61345261347531</v>
       </c>
+      <c r="T15" t="n">
+        <v>1651.29797979798</v>
+      </c>
+      <c r="U15" t="n">
+        <v>14.68976945053365</v>
+      </c>
+      <c r="V15" t="n">
+        <v>1535.722222222222</v>
+      </c>
+      <c r="W15" t="n">
+        <v>8.255445733813019</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1374,11 +1548,25 @@
       <c r="S16" t="n">
         <v>2.256464382135027</v>
       </c>
+      <c r="T16" t="n">
+        <v>1446.934343434343</v>
+      </c>
+      <c r="U16" t="n">
+        <v>4.532275893431197</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1396.217171717172</v>
+      </c>
+      <c r="W16" t="n">
+        <v>1.61913769567796</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="11">
     <mergeCell ref="N1:O1"/>
     <mergeCell ref="D1:E1"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="T1:U1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="L1:M1"/>
     <mergeCell ref="J1:K1"/>

</xml_diff>